<commit_message>
Fix context related problems
</commit_message>
<xml_diff>
--- a/docs/guni_qa_dataset.xlsx
+++ b/docs/guni_qa_dataset.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F77"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2088,9 +2088,85 @@
         <v>https://www.ganpatuniversity.ac.in/</v>
       </c>
     </row>
+    <row r="75" xml:space="preserve">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="str">
+        <v>How many streams are available at Ganpat University?</v>
+      </c>
+      <c r="C75" t="str" xml:space="preserve">
+        <v xml:space="preserve">Ganpat University offers academic programs across 8+ major faculties and streams:
+1. Engineering &amp; Technology (U.V. Patel College of Engineering - UVPCE): B.Tech, M.Tech, and Diploma in Computer Engineering, AI, Cyber Security, Mechanical, Civil, Electrical, and Biomedical.
+2. Management Studies (V.M. Patel Institute of Management - VMPIM): MBA, BBA, B.Com, and Executive Management.
+3. Computer Science &amp; Applications: BCA, MCA, B.Sc IT, M.Sc IT, and Cloud Computing.
+4. Pharmacy &amp; Healthcare (S.K. Patel College of Pharmaceutical Education &amp; Research - SKPCPER): B.Pharm, M.Pharm, and Pharm.D.
+5. Sciences (Mehsana Urban Institute of Sciences - MUIS): B.Sc and M.Sc in Biotechnology, Microbiology, Chemistry, Physics, and Mathematics.
+6. Agriculture &amp; Allied Sciences: B.Sc (Hons.) Agriculture approved as per ICAR guidelines.
+7. Marine Engineering &amp; Maritime Studies: DG Shipping approved maritime courses including Marine Engineering, GP Rating, and ETO.
+8. Healthcare, Nursing &amp; Physiotherapy: B.Sc Nursing, GNM, and Allied Health Sciences.</v>
+      </c>
+      <c r="D75" t="str">
+        <v>ACADEMIC &amp; PROGRAMS</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Academic Streams &amp; Faculties</v>
+      </c>
+      <c r="F75" t="str">
+        <v>https://www.ganpatuniversity.ac.in/admission</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="str">
+        <v>Which academic streams, courses and fields can I study at Ganpat University?</v>
+      </c>
+      <c r="C76" t="str">
+        <v>Ganpat University provides more than 150+ undergraduate (UG), postgraduate (PG), diploma, and doctoral (Ph.D.) degree programs across 8 core academic streams: Engineering &amp; Technology, Computer Applications, Management, Pharmacy, Applied Sciences, Agriculture, Marine Engineering, and Healthcare/Nursing.</v>
+      </c>
+      <c r="D76" t="str">
+        <v>ACADEMIC &amp; PROGRAMS</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Programs Overview</v>
+      </c>
+      <c r="F76" t="str">
+        <v>https://www.ganpatuniversity.ac.in/admission</v>
+      </c>
+    </row>
+    <row r="77" xml:space="preserve">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="str">
+        <v>How many faculties or departments are there at Ganpat University?</v>
+      </c>
+      <c r="C77" t="str" xml:space="preserve">
+        <v xml:space="preserve">Ganpat University comprises multiple prominent constituent faculties and institutes:
+- Faculty of Engineering &amp; Technology (UVPCE)
+- Faculty of Management Studies (VMPIM)
+- Faculty of Computer Applications
+- Faculty of Pharmacy (SKPCPER)
+- Faculty of Science (MUIS)
+- Faculty of Agriculture &amp; Allied Sciences
+- Marine Engineering &amp; Maritime Training Center
+- Faculty of Social Sciences, Humanities &amp; Nursing</v>
+      </c>
+      <c r="D77" t="str">
+        <v>ACADEMIC &amp; PROGRAMS</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Faculties &amp; Institutes</v>
+      </c>
+      <c r="F77" t="str">
+        <v>https://www.ganpatuniversity.ac.in/faculty</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F74"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F77"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>